<commit_message>
Public snapshot at REPORTPAGE-01
The full technical report at /report/; the showcase set, its charts and summary held to one run;
the schedule cross-check judged on the run's own basis. Cut from the tagged commit, CLEAN, client
gate green.
</commit_message>
<xml_diff>
--- a/templates/register_template.xlsx
+++ b/templates/register_template.xlsx
@@ -5675,7 +5675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B266"/>
+  <dimension ref="A1:B282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5946,1034 +5946,1034 @@
     <row r="42">
       <c r="A42" s="35" t="inlineStr">
         <is>
+          <t>from src.rng_streams import SEED_DRAWN, resolve_seed</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
           <t>from src.tier1_headless import METHODOLOGY_SHEET_TITLE, run_headless</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="35" t="n"/>
-    </row>
     <row r="44">
-      <c r="A44" s="35" t="inlineStr">
-        <is>
-          <t># ---------------------------------------------------------------------------</t>
-        </is>
-      </c>
+      <c r="A44" s="35" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="35" t="inlineStr">
         <is>
-          <t># xlwings Lite COMPATIBILITY (this class of defect cannot be caught headless)</t>
+          <t># ---------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="35" t="inlineStr">
         <is>
-          <t># ---------------------------------------------------------------------------</t>
+          <t># xlwings Lite COMPATIBILITY (this class of defect cannot be caught headless)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="35" t="inlineStr">
         <is>
-          <t># xlwings Lite's Office.js backend does NOT implement several classic xlwings</t>
+          <t># ---------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="35" t="inlineStr">
         <is>
-          <t># Sheet APIs. The Tier-1 shell MUST NOT use any of these (they raise a</t>
+          <t># xlwings Lite's Office.js backend does NOT implement several classic xlwings</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="35" t="inlineStr">
         <is>
-          <t># base-class NotImplementedError only at runtime in Excel - the headless gates</t>
+          <t># Sheet APIs. The Tier-1 shell MUST NOT use any of these (they raise a</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="35" t="inlineStr">
         <is>
-          <t># read via openpyxl and never exercise them):</t>
+          <t># base-class NotImplementedError only at runtime in Excel - the headless gates</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="35" t="inlineStr">
         <is>
-          <t>#</t>
+          <t># read via openpyxl and never exercise them):</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="35" t="inlineStr">
         <is>
-          <t>#   FORBIDDEN in Lite:  sheet.used_range   (xlwings-lite discussion #19)</t>
+          <t>#</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="35" t="inlineStr">
         <is>
-          <t>#                       sheet.copy()</t>
+          <t>#   FORBIDDEN in Lite:  sheet.used_range   (xlwings-lite discussion #19)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="35" t="inlineStr">
         <is>
-          <t>#                       sheet.api / Office.js getUsedRange (`.api` unsupported)</t>
+          <t>#                       sheet.copy()</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="35" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>#                       sheet.api / Office.js getUsedRange (`.api` unsupported)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="35" t="inlineStr">
         <is>
-          <t># SUPPORTED reads/writes used here: named ranges via book.names[nm].</t>
+          <t>#</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="35" t="inlineStr">
         <is>
-          <t># refers_to_range (Set_*, Out_*, Grid_RiskRegister, Grid_Methodology), and a FIXED</t>
+          <t># SUPPORTED reads/writes used here: named ranges via book.names[nm].</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="35" t="inlineStr">
         <is>
-          <t># A1-anchored address read via book.sheets[name].range("A1:..") (Office.js getRange -</t>
+          <t># refers_to_range (Set_*, Out_*, Grid_RiskRegister, Grid_Methodology), and a FIXED</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="35" t="inlineStr">
         <is>
-          <t># NOT getUsedRange). The grids are anchored at $A$1 (the parser uses ABSOLUTE Excel</t>
+          <t># A1-anchored address read via book.sheets[name].range("A1:..") (Office.js getRange -</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="35" t="inlineStr">
         <is>
-          <t># row indices, so the grid must be row-1-aligned).</t>
+          <t># NOT getUsedRange). The grids are anchored at $A$1 (the parser uses ABSOLUTE Excel</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="35" t="inlineStr">
         <is>
-          <t>#</t>
+          <t># row indices, so the grid must be row-1-aligned).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="35" t="inlineStr">
         <is>
-          <t># REG05-A2-FIX (D1): the Layer-1 sheets are read via their whole USED RANGE (a</t>
+          <t>#</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="35" t="inlineStr">
         <is>
-          <t># generous fixed A1 block, see _sheet_grid), NOT the fixed Grid_Layer1_* names. The</t>
+          <t># REG05-A2-FIX (D1): the Layer-1 sheets are read via their whole USED RANGE (a</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="35" t="inlineStr">
         <is>
-          <t># Grid_Layer1_* names are sized to the empty template's header-only shell and do NOT</t>
+          <t># generous fixed A1 block, see _sheet_grid), NOT the fixed Grid_Layer1_* names. The</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="35" t="inlineStr">
         <is>
-          <t># grow when the user fills the sheets, so a name-read saw only the shell (base sum</t>
+          <t># Grid_Layer1_* names are sized to the empty template's header-only shell and do NOT</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="35" t="inlineStr">
         <is>
-          <t># 3.9M != declared 50M, 0 factors, empty allocation). The used-range read grows with</t>
+          <t># grow when the user fills the sheets, so a name-read saw only the shell (base sum</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="35" t="inlineStr">
         <is>
-          <t># the fill and matches tier1_headless.extract_grids_openpyxl. The Grid_Layer1_* names</t>
+          <t># 3.9M != declared 50M, 0 factors, empty allocation). The used-range read grows with</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="35" t="inlineStr">
         <is>
-          <t># stay EMITTED (contract v1.4 / Validate) - a contract surface, just not the read</t>
+          <t># the fill and matches tier1_headless.extract_grids_openpyxl. The Grid_Layer1_* names</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
         <is>
-          <t># source. Not .expand() (truncates at the V5 layout's interior blank rows) and not</t>
+          <t># stay EMITTED (contract v1.4 / Validate) - a contract surface, just not the read</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="35" t="inlineStr">
         <is>
-          <t># .used_range/.api (Lite-forbidden); the parser trims trailing blanks, so an</t>
+          <t># source. Not .expand() (truncates at the V5 layout's interior blank rows) and not</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="35" t="inlineStr">
         <is>
-          <t># over-extended fixed block is harmless.</t>
+          <t># .used_range/.api (Lite-forbidden); the parser trims trailing blanks, so an</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="35" t="inlineStr">
         <is>
-          <t>_GRID_NAMES: dict[str, str] = {</t>
+          <t># over-extended fixed block is harmless.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    RISK_REGISTER_SHEET: "Grid_RiskRegister",</t>
+          <t>_GRID_NAMES: dict[str, str] = {</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    METHODOLOGY_SHEET_TITLE: "Grid_Methodology",</t>
+          <t xml:space="preserve">    RISK_REGISTER_SHEET: "Grid_RiskRegister",</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">    METHODOLOGY_SHEET_TITLE: "Grid_Methodology",</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="35" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="35" t="n"/>
-    </row>
     <row r="77">
-      <c r="A77" s="35" t="inlineStr">
-        <is>
-          <t># Fixed A1-anchored block for the Layer-1 used-range read (rows x cols). Must</t>
-        </is>
-      </c>
+      <c r="A77" s="35" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="35" t="inlineStr">
         <is>
-          <t># comfortably exceed any realistic Layer-1 extent (cost columns, WBS rows, factors -</t>
+          <t># Fixed A1-anchored block for the Layer-1 used-range read (rows x cols). Must</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="35" t="inlineStr">
         <is>
-          <t># a compact factor model, never a large table); the parser trims trailing blanks.</t>
+          <t># comfortably exceed any realistic Layer-1 extent (cost columns, WBS rows, factors -</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="35" t="inlineStr">
         <is>
-          <t># Parked robust option (brief §2.1): dynamic OFFSET Grid_Layer1_* names.</t>
+          <t># a compact factor model, never a large table); the parser trims trailing blanks.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="35" t="inlineStr">
         <is>
+          <t># Parked robust option (brief §2.1): dynamic OFFSET Grid_Layer1_* names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="35" t="inlineStr">
+        <is>
           <t>_LAYER1_READ_RANGE = "A1:AX200"  # AX = col 50; 200 rows</t>
         </is>
       </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="35" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="35" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="35" t="inlineStr">
-        <is>
-          <t>def _range_grid(book, range_name: str):</t>
-        </is>
-      </c>
+      <c r="A84" s="35" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Read a named range's values as a 2D grid (list of row-lists). Returns []</t>
+          <t>def _range_grid(book, range_name: str):</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if the named range is absent. Lite-safe (named-range read only)."""</t>
+          <t xml:space="preserve">    """Read a named range's values as a 2D grid (list of row-lists). Returns []</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    try:</t>
+          <t xml:space="preserve">    if the named range is absent. Lite-safe (named-range read only)."""</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        rng = book.names[range_name].refers_to_range</t>
+          <t xml:space="preserve">    try:</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    except (KeyError, Exception):  # noqa: BLE001 - Lite raises varied types on a missing name</t>
+          <t xml:space="preserve">        rng = book.names[range_name].refers_to_range</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return []</t>
+          <t xml:space="preserve">    except (KeyError, Exception):  # noqa: BLE001 - Lite raises varied types on a missing name</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    v = rng.value</t>
+          <t xml:space="preserve">        return []</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if v is None:</t>
+          <t xml:space="preserve">    v = rng.value</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return []</t>
+          <t xml:space="preserve">    if v is None:</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if not isinstance(v, list):</t>
+          <t xml:space="preserve">        return []</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return [[v]]  # single cell</t>
+          <t xml:space="preserve">    if not isinstance(v, list):</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if v and not isinstance(v[0], list):</t>
+          <t xml:space="preserve">        return [[v]]  # single cell</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        v = [v]  # xlwings collapses a single row to 1D; re-wrap to 2D</t>
+          <t xml:space="preserve">    if v and not isinstance(v[0], list):</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">        v = [v]  # xlwings collapses a single row to 1D; re-wrap to 2D</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">    return v</t>
         </is>
       </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="35" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="35" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="35" t="inlineStr">
-        <is>
-          <t>def _sheet_grid(book, sheet_name: str):</t>
-        </is>
-      </c>
+      <c r="A101" s="35" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Read a whole Layer-1 sheet as a 2D grid over a generous FIXED A1-anchored</t>
+          <t>def _sheet_grid(book, sheet_name: str):</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    block (:data:`_LAYER1_READ_RANGE`). Lite-safe: an explicit address via</t>
+          <t xml:space="preserve">    """Read a whole Layer-1 sheet as a 2D grid over a generous FIXED A1-anchored</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ``book.sheets[name].range(addr)`` (Office.js getRange), never the Lite-forbidden</t>
+          <t xml:space="preserve">    block (:data:`_LAYER1_READ_RANGE`). Lite-safe: an explicit address via</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    whole-sheet readers listed in this module's header. Grows with the user's fill</t>
+          <t xml:space="preserve">    ``book.sheets[name].range(addr)`` (Office.js getRange), never the Lite-forbidden</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    where the fixed ``Grid_Layer1_*`` name would not (REG05-A2-FIX D1); the parser</t>
+          <t xml:space="preserve">    whole-sheet readers listed in this module's header. Grows with the user's fill</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    trims trailing blanks, so over-covering is harmless. ``[]`` if the sheet absent."""</t>
+          <t xml:space="preserve">    where the fixed ``Grid_Layer1_*`` name would not (REG05-A2-FIX D1); the parser</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    try:</t>
+          <t xml:space="preserve">    trims trailing blanks, so over-covering is harmless. ``[]`` if the sheet absent."""</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        sht = book.sheets[sheet_name]</t>
+          <t xml:space="preserve">    try:</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    except (KeyError, Exception):  # noqa: BLE001 - Lite raises varied types when absent</t>
+          <t xml:space="preserve">        sht = book.sheets[sheet_name]</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return []</t>
+          <t xml:space="preserve">    except (KeyError, Exception):  # noqa: BLE001 - Lite raises varied types when absent</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    try:</t>
+          <t xml:space="preserve">        return []</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        v = sht.range(_LAYER1_READ_RANGE).value</t>
+          <t xml:space="preserve">    try:</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    except Exception:  # noqa: BLE001 - a missing/empty sheet range reads as nothing</t>
+          <t xml:space="preserve">        v = sht.range(_LAYER1_READ_RANGE).value</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return []</t>
+          <t xml:space="preserve">    except Exception:  # noqa: BLE001 - a missing/empty sheet range reads as nothing</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if v is None:</t>
+          <t xml:space="preserve">        return []</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return []</t>
+          <t xml:space="preserve">    if v is None:</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if not isinstance(v, list):</t>
+          <t xml:space="preserve">        return []</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        v = [[v]]                       # single cell</t>
+          <t xml:space="preserve">    if not isinstance(v, list):</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    elif v and not isinstance(v[0], list):</t>
+          <t xml:space="preserve">        v = [[v]]                       # single cell</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        v = [v]                         # xlwings collapses a single row to 1D</t>
+          <t xml:space="preserve">    elif v and not isinstance(v[0], list):</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # trim trailing all-blank rows so the grid matches the openpyxl used range.</t>
+          <t xml:space="preserve">        v = [v]                         # xlwings collapses a single row to 1D</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    while v and all(c is None for c in v[-1]):</t>
+          <t xml:space="preserve">    # trim trailing all-blank rows so the grid matches the openpyxl used range.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        v.pop()</t>
+          <t xml:space="preserve">    while v and all(c is None for c in v[-1]):</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">        v.pop()</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">    return v</t>
         </is>
       </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="35" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="35" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="35" t="inlineStr">
-        <is>
-          <t>def read_grids_xlwings(book) -&gt; dict:</t>
-        </is>
-      </c>
+      <c r="A128" s="35" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Tier-1 grid extraction (the Lite-safe analogue of</t>
+          <t>def read_grids_xlwings(book) -&gt; dict:</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ``tier1_headless.extract_grids_openpyxl``). Risk register + methodology via their</t>
+          <t xml:space="preserve">    """Tier-1 grid extraction (the Lite-safe analogue of</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ``Grid_*`` named ranges (sized to extent at build); the Layer-1 sheets via their</t>
+          <t xml:space="preserve">    ``tier1_headless.extract_grids_openpyxl``). Risk register + methodology via their</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    whole USED RANGE (:func:`_sheet_grid`, REG05-A2-FIX D1). Same grids, same parser.</t>
+          <t xml:space="preserve">    ``Grid_*`` named ranges (sized to extent at build); the Layer-1 sheets via their</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">    whole USED RANGE (:func:`_sheet_grid`, REG05-A2-FIX D1). Same grids, same parser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">    A client register with no Layer-1 sheets -&gt; ``layer1={}`` -&gt; Layer 1 OFF, as Tier 2.</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="35" t="n"/>
-    </row>
     <row r="135">
-      <c r="A135" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    REG05-A2 §3.2: read ``Set_Layer1_Enabled`` and thread it in as</t>
-        </is>
-      </c>
+      <c r="A135" s="35" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ``layer1_enabled``; when not TRUE, pass ``layer1={}`` so the shared parse gate</t>
+          <t xml:space="preserve">    REG05-A2 §3.2: read ``Set_Layer1_Enabled`` and thread it in as</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    returns None (an empty, present-but-disabled Layer-1 is a read no-op)."""</t>
+          <t xml:space="preserve">    ``layer1_enabled``; when not TRUE, pass ``layer1={}`` so the shared parse gate</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    enabled = layer1_enabled_flag(_named_value(book, LAYER1_ENABLED_NAME))</t>
+          <t xml:space="preserve">    returns None (an empty, present-but-disabled Layer-1 is a read no-op)."""</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    layer1 = (</t>
+          <t xml:space="preserve">    enabled = layer1_enabled_flag(_named_value(book, LAYER1_ENABLED_NAME))</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">    layer1 = (</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            sheet: _sheet_grid(book, sheet)</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            for sheet in _LAYER1_SHEETS</t>
+          <t xml:space="preserve">            sheet: _sheet_grid(book, sheet)</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if _sheet_grid(book, sheet)</t>
+          <t xml:space="preserve">            for sheet in _LAYER1_SHEETS</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">            if _sheet_grid(book, sheet)</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if enabled else {}</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    )</t>
+          <t xml:space="preserve">        if enabled else {}</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    return {</t>
+          <t xml:space="preserve">    )</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "risk_register": _range_grid(book, _GRID_NAMES[RISK_REGISTER_SHEET]),</t>
+          <t xml:space="preserve">    return {</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "layer1": layer1,</t>
+          <t xml:space="preserve">        "risk_register": _range_grid(book, _GRID_NAMES[RISK_REGISTER_SHEET]),</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "layer1_enabled": enabled,</t>
+          <t xml:space="preserve">        "layer1": layer1,</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        # GD-B: the register's own methodology surface (CG coeffs + mode</t>
+          <t xml:space="preserve">        "layer1_enabled": enabled,</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        # multipliers). Absent -&gt; [] -&gt; the resolver fails loud (no fallback).</t>
+          <t xml:space="preserve">        # GD-B: the register's own methodology surface (CG coeffs + mode</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "methodology": _range_grid(book, _GRID_NAMES[METHODOLOGY_SHEET_TITLE]),</t>
+          <t xml:space="preserve">        # multipliers). Absent -&gt; [] -&gt; the resolver fails loud (no fallback).</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">        "methodology": _range_grid(book, _GRID_NAMES[METHODOLOGY_SHEET_TITLE]),</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">    }</t>
         </is>
       </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="35" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="35" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="35" t="inlineStr">
-        <is>
-          <t>def _named_value(book, name):</t>
-        </is>
-      </c>
+      <c r="A157" s="35" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Read a named-range scalar value (Lite-safe). Returns None if absent."""</t>
+          <t>def _named_value(book, name):</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    try:</t>
+          <t xml:space="preserve">    """Read a named-range scalar value (Lite-safe). Returns None if absent."""</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return book.names[name].refers_to_range.value</t>
+          <t xml:space="preserve">    try:</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    except Exception:  # noqa: BLE001 - Lite raises varied types on a missing name</t>
+          <t xml:space="preserve">        return book.names[name].refers_to_range.value</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">    except Exception:  # noqa: BLE001 - Lite raises varied types on a missing name</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">        return None</t>
         </is>
       </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="35" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="35" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="35" t="inlineStr">
-        <is>
-          <t>def _pad(rows2d: list, nrows: int, ncols: int) -&gt; list:</t>
-        </is>
-      </c>
+      <c r="A165" s="35" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Truncate/pad a 2D list to (nrows, ncols) with None so the write matches</t>
+          <t>def _pad(rows2d: list, nrows: int, ncols: int) -&gt; list:</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    the fixed named-range shape (RF-01 pattern)."""</t>
+          <t xml:space="preserve">    """Truncate/pad a 2D list to (nrows, ncols) with None so the write matches</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    out = []</t>
+          <t xml:space="preserve">    the fixed named-range shape (RF-01 pattern)."""</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for i in range(nrows):</t>
+          <t xml:space="preserve">    out = []</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        row = list(rows2d[i]) if i &lt; len(rows2d) else []</t>
+          <t xml:space="preserve">    for i in range(nrows):</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        out.append([(row[j] if j &lt; len(row) else None) for j in range(ncols)])</t>
+          <t xml:space="preserve">        row = list(rows2d[i]) if i &lt; len(rows2d) else []</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">        out.append([(row[j] if j &lt; len(row) else None) for j in range(ncols)])</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">    return out</t>
         </is>
       </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="35" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="35" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="35" t="inlineStr">
-        <is>
-          <t>def _run_and_write(book, iterations_name: str, default_iter: int):</t>
-        </is>
-      </c>
+      <c r="A175" s="35" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Shared run path for the run buttons: read Set_* ranges -&gt; run_headless -&gt;</t>
+          <t>def _run_and_write(book, iterations_name: str, default_iter: int):</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    write Out_* ranges. ``iterations_name`` selects which Settings cell drives the</t>
+          <t xml:space="preserve">    """Shared run path for the run buttons: read Set_* ranges -&gt; run_headless -&gt;</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    iteration count (Set_iterations = interactive default; Set_iterations_max =</t>
+          <t xml:space="preserve">    write Out_* ranges. ``iterations_name`` selects which Settings cell drives the</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    the 100k button). Named-range reads/writes only (Lite-safe)."""</t>
+          <t xml:space="preserve">    iteration count (Set_iterations = interactive default; Set_iterations_max =</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">    the 100k button). Named-range reads/writes only (Lite-safe)."""</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">    grids = read_grids_xlwings(book)</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="35" t="n"/>
-    </row>
     <row r="182">
-      <c r="A182" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    def R(nm):</t>
-        </is>
-      </c>
+      <c r="A182" s="35" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">    def R(nm):</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">        return book.names[nm].refers_to_range</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="35" t="n"/>
-    </row>
     <row r="185">
-      <c r="A185" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    def _named(nm, default):</t>
-        </is>
-      </c>
+      <c r="A185" s="35" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        try:</t>
+          <t xml:space="preserve">    def _named(nm, default):</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            return R(nm).value</t>
+          <t xml:space="preserve">        try:</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        except Exception:</t>
+          <t xml:space="preserve">            return R(nm).value</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="35" t="inlineStr">
         <is>
+          <t xml:space="preserve">        except Exception:</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="35" t="inlineStr">
+        <is>
           <t xml:space="preserve">            return default</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="35" t="n"/>
-    </row>
     <row r="191">
-      <c r="A191" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    n_iter = int(_named(iterations_name, default_iter) or default_iter)</t>
-        </is>
-      </c>
+      <c r="A191" s="35" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    seed = int(_named("Set_seed", 42) or 42)</t>
+          <t xml:space="preserve">    n_iter = int(_named(iterations_name, default_iter) or default_iter)</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    view = str(_named("Set_view", "owner") or "owner").strip().lower()</t>
+          <t xml:space="preserve">    # SEEDZERO-01 P5: a stated seed is used as given; blank or 0 is drawn here and written back</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # GENERIC-01: no fallback. `Set_risk_prefix` is contract-required, and defaulting it to the</t>
+          <t xml:space="preserve">    # below, so the workbook records the seed its outputs came from. A fraction is refused, not</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # wind project's "WT" meant a register that omitted it had every risk row read against another</t>
+          <t xml:space="preserve">    # truncated. The range is contract-required: without it a drawn seed has nowhere to be</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # project's prefix, matched none, and returned an EMPTY result rather than an error - a wrong</t>
+          <t xml:space="preserve">    # recorded, so a missing one is refused rather than run unrecorded.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # answer where the missing range should have been a refusal.</t>
+          <t xml:space="preserve">    try:</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    prefix = str(_named("Set_risk_prefix", "") or "").strip()</t>
+          <t xml:space="preserve">        seed_range = R("Set_seed")</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if not prefix:</t>
+          <t xml:space="preserve">    except Exception:</t>
         </is>
       </c>
     </row>
@@ -6987,153 +6987,157 @@
     <row r="201">
       <c r="A201" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "Set_risk_prefix is missing or empty. It is required by the register contract and "</t>
+          <t xml:space="preserve">            "Set_seed is missing. It is required by the register contract, and it is where a "</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "there is no default: a prefix borrowed from another project would match no risk "</t>
+          <t xml:space="preserve">            "drawn seed is recorded: restore it (Settings!B2), blank or 0 for a random run."</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "rows and report an empty register as though it were a result.")</t>
+          <t xml:space="preserve">        ) from None</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="35" t="n"/>
+      <c r="A204" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    seed, seed_source = resolve_seed(seed_range.value, where="Set_seed")</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # The ENTIRE compute + formatting is the headless core (CI-covered). This</t>
+          <t xml:space="preserve">    view = str(_named("Set_view", "owner") or "owner").strip().lower()</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # wrapper only reads the ranges above and writes the ranges below.</t>
+          <t xml:space="preserve">    # GENERIC-01: no fallback. `Set_risk_prefix` is contract-required, and defaulting it to the</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    out = run_headless(grids, risk_id_prefix=prefix, n_iter=n_iter, seed=seed, view=view)</t>
+          <t xml:space="preserve">    # wind project's "WT" meant a register that omitted it had every risk row read against another</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="35" t="n"/>
+      <c r="A208" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    # project's prefix, matched none, and returned an EMPTY result rather than an error - a wrong</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R("Out_ptable").value = _pad(out["p_table"], 19, 2)</t>
+          <t xml:space="preserve">    # answer where the missing range should have been a refusal.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R("Out_scurve").value = _pad(</t>
+          <t xml:space="preserve">    prefix = str(_named("Set_risk_prefix", "") or "").strip()</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        list(zip(out["s_curve"]["prob"], out["s_curve"]["value"])), 101, 2</t>
+          <t xml:space="preserve">    if not prefix:</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    )</t>
+          <t xml:space="preserve">        raise ValueError(</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R("Corr_flag").value = out["corr_flag"]</t>
+          <t xml:space="preserve">            "Set_risk_prefix is missing or empty. It is required by the register contract and "</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    conv = out["convergence_note"]</t>
+          <t xml:space="preserve">            "there is no default: a prefix borrowed from another project would match no risk "</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R("Out_conv_halfwidth").value = round(conv["p80_ci95_half_width"], 2)</t>
+          <t xml:space="preserve">            "rows and report an empty register as though it were a result.")</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    R("Out_conv_pct").value = round(conv["p80_ci95_half_width_pct"], 4)</t>
-        </is>
-      </c>
+      <c r="A216" s="35" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if out["triple"]:</t>
+          <t xml:space="preserve">    # The ENTIRE compute + formatting is the headless core (CI-covered). This</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        modes = ("zero", "elicited", "one")</t>
+          <t xml:space="preserve">    # wrapper only reads the ranges above and writes the ranges below.</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        triple_rows = [</t>
+          <t xml:space="preserve">    out = run_headless(grids, risk_id_prefix=prefix, n_iter=n_iter, seed=seed, view=view)</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            [out["triple"]["elicited"][i][0]] + [out["triple"][m][i][1] for m in modes]</t>
+          <t xml:space="preserve">    # First write: if a later output write fails, the outputs already in the sheet still name</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            for i in range(len(out["triple"]["elicited"]))</t>
+          <t xml:space="preserve">    # the seed they came from.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ]</t>
+          <t xml:space="preserve">    if seed_source == SEED_DRAWN:</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        R("Out_triple").value = _pad(triple_rows, 19, 4)</t>
+          <t xml:space="preserve">        seed_range.value = seed</t>
         </is>
       </c>
     </row>
@@ -7141,197 +7145,201 @@
       <c r="A224" s="35" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="35" t="n"/>
+      <c r="A225" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    R("Out_ptable").value = _pad(out["p_table"], 19, 2)</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="35" t="inlineStr">
         <is>
-          <t>@script</t>
+          <t xml:space="preserve">    R("Out_scurve").value = _pad(</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="35" t="inlineStr">
         <is>
-          <t>def run_simulation(book: xw.Book):  # pragma: no cover - exercised in Excel (6b load test)</t>
+          <t xml:space="preserve">        list(zip(out["s_curve"]["prob"], out["s_curve"]["value"])), 101, 2</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """BUTTON: run the cost-QRA at the interactive iteration count (Settings B1 /</t>
+          <t xml:space="preserve">    )</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Set_iterations, default 25k) and write the P-curve/S-curve/convergence back."""</t>
+          <t xml:space="preserve">    R("Corr_flag").value = out["corr_flag"]</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    _run_and_write(book, "Set_iterations", 25_000)</t>
+          <t xml:space="preserve">    conv = out["convergence_note"]</t>
         </is>
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="35" t="n"/>
+      <c r="A231" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    R("Out_conv_halfwidth").value = round(conv["p80_ci95_half_width"], 2)</t>
+        </is>
+      </c>
     </row>
     <row r="232">
-      <c r="A232" s="35" t="n"/>
+      <c r="A232" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    R("Out_conv_pct").value = round(conv["p80_ci95_half_width_pct"], 4)</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="35" t="inlineStr">
         <is>
-          <t>@script</t>
+          <t xml:space="preserve">    if out["triple"]:</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="35" t="inlineStr">
         <is>
-          <t>def run_simulation_100k(book: xw.Book):  # pragma: no cover - exercised in Excel</t>
+          <t xml:space="preserve">        modes = ("zero", "elicited", "one")</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """BUTTON: run the cost-QRA at the on-demand 100k count (Settings B5 /</t>
+          <t xml:space="preserve">        triple_rows = [</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Set_iterations_max, default 100k) - the high-resolution run for the deliverable.</t>
+          <t xml:space="preserve">            [out["triple"]["elicited"][i][0]] + [out["triple"][m][i][1] for m in modes]</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Same write-back as run_simulation; only the iteration count differs."""</t>
+          <t xml:space="preserve">            for i in range(len(out["triple"]["elicited"]))</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    _run_and_write(book, "Set_iterations_max", 100_000)</t>
+          <t xml:space="preserve">        ]</t>
         </is>
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="35" t="n"/>
+      <c r="A239" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        R("Out_triple").value = _pad(triple_rows, 19, 4)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="35" t="n"/>
     </row>
     <row r="241">
-      <c r="A241" s="35" t="inlineStr">
-        <is>
-          <t>@script</t>
-        </is>
-      </c>
+      <c r="A241" s="35" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="35" t="inlineStr">
         <is>
-          <t>def validate_contract(book: xw.Book):  # pragma: no cover - exercised in Excel</t>
+          <t>@script</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """REG03 S2 rider (1): a contract self-check for a scaffold-once handover.</t>
+          <t>def run_simulation(book: xw.Book):  # pragma: no cover - exercised in Excel (6b load test)</t>
         </is>
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="35" t="n"/>
+      <c r="A244" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    """BUTTON: run the cost-QRA at the interactive iteration count (Settings B1 /</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    After a user hand-edits the scaffolded register, this verifies the</t>
+          <t xml:space="preserve">    Set_iterations, default 25k) and write the P-curve/S-curve/convergence back."""</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Grid_*/Set_*/Out_* named ranges are all present, Set_ContractVersion matches,</t>
+          <t xml:space="preserve">    _run_and_write(book, "Set_iterations", 25_000)</t>
         </is>
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    and Grid_Methodology carries its 13 CG + 3 mode rows - writing PASS/FAIL + a</t>
-        </is>
-      </c>
+      <c r="A247" s="35" t="n"/>
     </row>
     <row r="248">
-      <c r="A248" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    human-readable message to the Out_validation range. A thin I/O wrapper over the</t>
-        </is>
-      </c>
+      <c r="A248" s="35" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    headless ``check_contract`` (CI-covered); it reads via named ranges only, so it</t>
+          <t>@script</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    obeys the Lite forbidden-API list documented in this module's header."""</t>
+          <t>def run_simulation_100k(book: xw.Book):  # pragma: no cover - exercised in Excel</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    grids = read_grids_xlwings(book)</t>
+          <t xml:space="preserve">    """BUTTON: run the cost-QRA at the on-demand 100k count (Settings B5 /</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    try:</t>
+          <t xml:space="preserve">    Set_iterations_max, default 100k) - the high-resolution run for the deliverable.</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        present = [nm.name for nm in book.names]</t>
+          <t xml:space="preserve">    Same write-back as run_simulation; only the iteration count differs."""</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    except Exception:</t>
+          <t xml:space="preserve">    _run_and_write(book, "Set_iterations_max", 100_000)</t>
         </is>
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        present = []</t>
-        </is>
-      </c>
+      <c r="A255" s="35" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="35" t="n"/>
@@ -7339,64 +7347,168 @@
     <row r="257">
       <c r="A257" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    def _named(nm, default=None):</t>
+          <t>@script</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        try:</t>
+          <t>def validate_contract(book: xw.Book):  # pragma: no cover - exercised in Excel</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            return book.names[nm].refers_to_range.value</t>
+          <t xml:space="preserve">    """REG03 S2 rider (1): a contract self-check for a scaffold-once handover.</t>
         </is>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        except Exception:</t>
-        </is>
-      </c>
+      <c r="A260" s="35" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">            return default</t>
+          <t xml:space="preserve">    After a user hand-edits the scaffolded register, this verifies the</t>
         </is>
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="35" t="n"/>
+      <c r="A262" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Grid_*/Set_*/Out_* named ranges are all present, Set_ContractVersion matches,</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ok, message = check_contract(present, grids["methodology"],</t>
+          <t xml:space="preserve">    and Grid_Methodology carries its 13 CG + 3 mode rows - writing PASS/FAIL + a</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                 _named("Set_ContractVersion"))</t>
+          <t xml:space="preserve">    human-readable message to the Out_validation range. A thin I/O wrapper over the</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    book.names["Out_validation"].refers_to_range.value = [</t>
+          <t xml:space="preserve">    headless ``check_contract`` (CI-covered); it reads via named ranges only, so it</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    obeys the Lite forbidden-API list documented in this module's header."""</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    grids = read_grids_xlwings(book)</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    try:</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        present = [nm.name for nm in book.names]</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    except Exception:</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        present = []</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="35" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    def _named(nm, default=None):</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        try:</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            return book.names[nm].refers_to_range.value</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        except Exception:</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            return default</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="35" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ok, message = check_contract(present, grids["methodology"],</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                 _named("Set_ContractVersion"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    book.names["Out_validation"].refers_to_range.value = [</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">        ["PASS" if ok else "FAIL"], [message]]</t>
         </is>

</xml_diff>

<commit_message>
Public snapshot at INTSCURVE-01
</commit_message>
<xml_diff>
--- a/templates/register_template.xlsx
+++ b/templates/register_template.xlsx
@@ -1737,12 +1737,19 @@
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>RECORDED, NOT READ. Effectiveness_Confidence, Default_Mapping_Confidence and Assignment_Confidence are kept for a reviewer and never used by the engine: any scale, or blank.</t>
+          <t>COST IMPACT AND DELAY. Risk cost impacts exclude project time-related costs (preliminaries and site overheads). The model prices those once, through the day rate, on the finish delay that survives float in each iteration. Event-specific standby (idle plant or crew, demobilise / remobilise) is a direct cost and stays in the risk's cost impact. The day rate itself covers preliminaries and site overheads only, with no standby, so the same cost cannot enter through both the day rate and a risk's cost impact.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
+        <is>
+          <t>RECORDED, NOT READ. Effectiveness_Confidence, Default_Mapping_Confidence and Assignment_Confidence are kept for a reviewer and never used by the engine: any scale, or blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
         <is>
           <t>WHERE THE REST IS. Each fillable sheet carries its notes above its headers and each column's format on its header cell (hover). How to run: 'Running a simulation' above. What the colours mean: the legend above.</t>
         </is>

</xml_diff>